<commit_message>
Add ride share simulation script and total revenue calculation
- Implemented a comprehensive simulation for ride-sharing models including RR, RGD, SFB, AGM, and OPGD.
- Added functionality to generate and save total revenue statistics for different models and parameters.
- Created visualizations for prices, demand, individual revenues, and total revenues across multiple experiments.
- Introduced data handling for average and variance calculations, saving results to an Excel file for further analysis.
- Included necessary imports and utility functions for matrix generation and plotting.
</commit_message>
<xml_diff>
--- a/ride_share/figs/total_revenue.xlsx
+++ b/ride_share/figs/total_revenue.xlsx
@@ -463,22 +463,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>226089</t>
+          <t>226089 $\pm$ 0.00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>213894</t>
+          <t>213894 $\pm$ 0.00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>207620</t>
+          <t>207620 $\pm$ 0.00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>203429</t>
+          <t>203429 $\pm$ 0.00</t>
         </is>
       </c>
     </row>
@@ -490,22 +490,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>222839</t>
+          <t>222839 $\pm$ 472122.94</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>171981</t>
+          <t>171981 $\pm$ 752331.66</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>140523</t>
+          <t>140523 $\pm$ 1035136.32</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>118188</t>
+          <t>118188 $\pm$ 1137432.96</t>
         </is>
       </c>
     </row>
@@ -517,22 +517,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>222283</t>
+          <t>222283 $\pm$ 457555.72</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>169300</t>
+          <t>169300 $\pm$ 640906.85</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>136671</t>
+          <t>136671 $\pm$ 813603.90</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>113543</t>
+          <t>113543 $\pm$ 850454.77</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>220086</t>
+          <t>220086 $\pm$ 628761.50</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>161349</t>
+          <t>161349 $\pm$ 1437581.02</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>130896</t>
+          <t>130896 $\pm$ 2792420.94</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>113393</t>
+          <t>113393 $\pm$ 3839473.44</t>
         </is>
       </c>
     </row>
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>218509</t>
+          <t>218509 $\pm$ 669930.19</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>155989</t>
+          <t>155989 $\pm$ 1886652.94</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>121859</t>
+          <t>121859 $\pm$ 2875477.12</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>99987</t>
+          <t>99987 $\pm$ 3229487.34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update total revenue figures and improve noise handling in simulation
</commit_message>
<xml_diff>
--- a/ride_share/figs/total_revenue.xlsx
+++ b/ride_share/figs/total_revenue.xlsx
@@ -463,22 +463,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>226089 $\pm$ 0.00</t>
+          <t>219706 $\pm$ 257</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>213894 $\pm$ 0.00</t>
+          <t>213894 $\pm$ 0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>207620 $\pm$ 0.00</t>
+          <t>207620 $\pm$ 0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>203429 $\pm$ 0.00</t>
+          <t>203429 $\pm$ 0</t>
         </is>
       </c>
     </row>
@@ -490,22 +490,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>222839 $\pm$ 472122.94</t>
+          <t>214788 $\pm$ 1464</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>171981 $\pm$ 752331.66</t>
+          <t>165102 $\pm$ 0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>140523 $\pm$ 1035136.32</t>
+          <t>129945 $\pm$ 0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>118188 $\pm$ 1137432.96</t>
+          <t>104928 $\pm$ 0</t>
         </is>
       </c>
     </row>
@@ -517,22 +517,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>222283 $\pm$ 457555.72</t>
+          <t>213908 $\pm$ 1455</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>169300 $\pm$ 640906.85</t>
+          <t>162535 $\pm$ 0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>136671 $\pm$ 813603.90</t>
+          <t>126469 $\pm$ 0</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>113543 $\pm$ 850454.77</t>
+          <t>100936 $\pm$ 0</t>
         </is>
       </c>
     </row>
@@ -544,22 +544,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>220086 $\pm$ 628761.50</t>
+          <t>210471 $\pm$ 1773</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>161349 $\pm$ 1437581.02</t>
+          <t>154251 $\pm$ 0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>130896 $\pm$ 2792420.94</t>
+          <t>120459 $\pm$ 0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>113393 $\pm$ 3839473.44</t>
+          <t>101116 $\pm$ 0</t>
         </is>
       </c>
     </row>
@@ -571,22 +571,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>218509 $\pm$ 669930.19</t>
+          <t>208363 $\pm$ 1961</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>155989 $\pm$ 1886652.94</t>
+          <t>147491 $\pm$ 0</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>121859 $\pm$ 2875477.12</t>
+          <t>109373 $\pm$ 0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>99987 $\pm$ 3229487.34</t>
+          <t>85426 $\pm$ 0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update run_experiment flag to enable experiment execution in multiple scripts
</commit_message>
<xml_diff>
--- a/ride_share/figs/total_revenue.xlsx
+++ b/ride_share/figs/total_revenue.xlsx
@@ -463,22 +463,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>224556 $\pm$ 1186</t>
+          <t>228348 $\pm$ 664</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>217440 $\pm$ 834</t>
+          <t>219390 $\pm$ 723</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>214132 $\pm$ 1503</t>
+          <t>217054 $\pm$ 954</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>210790 $\pm$ 1336</t>
+          <t>214854 $\pm$ 780</t>
         </is>
       </c>
     </row>

</xml_diff>